<commit_message>
Rearmo commits sin el archivo pesado
</commit_message>
<xml_diff>
--- a/graficos/evasion/contribuciones_mca_2020.xlsx
+++ b/graficos/evasion/contribuciones_mca_2020.xlsx
@@ -26,10 +26,10 @@
     <t xml:space="preserve">Quality of representation</t>
   </si>
   <si>
-    <t xml:space="preserve">Contribution (left)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contribution (right)</t>
+    <t xml:space="preserve">Contribution (negative side)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contribution (positive side)</t>
   </si>
   <si>
     <t xml:space="preserve">Total contribution</t>

</xml_diff>